<commit_message>
reporte de maderera y modo celular para maderera
</commit_message>
<xml_diff>
--- a/public/formats/items.xlsx
+++ b/public/formats/items.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\laragon\www\sdrimsac-tenant\public\formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sdrimsac\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33928128-2A3B-42A2-AF0D-C3ABAAA665BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -206,7 +207,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -525,7 +526,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AR2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>

</xml_diff>

<commit_message>
buscador por marca modelo y calidad en caja subir por excel ubicacion modelo
</commit_message>
<xml_diff>
--- a/public/formats/items.xlsx
+++ b/public/formats/items.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sdrimsac\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33928128-2A3B-42A2-AF0D-C3ABAAA665BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD8D6FFE-0602-41D0-B639-24B96D2D75E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="67">
   <si>
     <t>Descripción</t>
   </si>
@@ -202,6 +202,30 @@
   </si>
   <si>
     <t>PRODUCTO PRUEBA TRATAMIENTO</t>
+  </si>
+  <si>
+    <t>ubicación</t>
+  </si>
+  <si>
+    <t>modelo</t>
+  </si>
+  <si>
+    <t>calidad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">codigo origen </t>
+  </si>
+  <si>
+    <t>XR</t>
+  </si>
+  <si>
+    <t>ORIGINAL</t>
+  </si>
+  <si>
+    <t>12345XZ</t>
+  </si>
+  <si>
+    <t>TIENDA 1</t>
   </si>
 </sst>
 </file>
@@ -527,7 +551,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR2"/>
+  <dimension ref="A1:AV2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -552,9 +576,10 @@
     <col min="39" max="39" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="41" max="41" width="13.85546875" bestFit="1" customWidth="1"/>
     <col min="43" max="43" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="48" max="48" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -687,8 +712,20 @@
       <c r="AR1" t="s">
         <v>49</v>
       </c>
+      <c r="AS1" t="s">
+        <v>59</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>60</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>61</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>62</v>
+      </c>
     </row>
-    <row r="2" spans="1:44" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:48" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -805,6 +842,18 @@
       </c>
       <c r="AN2">
         <v>13</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>66</v>
+      </c>
+      <c r="AT2" t="s">
+        <v>63</v>
+      </c>
+      <c r="AU2" t="s">
+        <v>64</v>
+      </c>
+      <c r="AV2" t="s">
+        <v>65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
peso en el excel de items
</commit_message>
<xml_diff>
--- a/public/formats/items.xlsx
+++ b/public/formats/items.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25601"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\laragon\www\sdrimsac-tenant\public\formats\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sdrimsac\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99FB8380-C83B-4B8E-9540-A3DC8395B30E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="70">
   <si>
     <t>Descripción</t>
   </si>
@@ -231,12 +232,15 @@
   </si>
   <si>
     <t>Talla/Colores</t>
+  </si>
+  <si>
+    <t>peso</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -555,8 +559,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AX2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:AY2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -584,7 +588,7 @@
     <col min="50" max="50" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -735,8 +739,11 @@
       <c r="AX1" t="s">
         <v>62</v>
       </c>
+      <c r="AY1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="2" spans="1:50" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:51" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -871,6 +878,9 @@
       </c>
       <c r="AX2" t="s">
         <v>65</v>
+      </c>
+      <c r="AY2">
+        <v>10</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
correcion de limpieza hotel
</commit_message>
<xml_diff>
--- a/public/formats/items.xlsx
+++ b/public/formats/items.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\sdrimsac\public\formats\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{253A1184-EE20-4058-B60D-BCE4649B9110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CAF78E92-3D35-4A46-A78A-816730BBFCFB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="76">
   <si>
     <t>Descripción</t>
   </si>
@@ -253,24 +253,6 @@
   </si>
   <si>
     <t>BG</t>
-  </si>
-  <si>
-    <t>Categortia Compra</t>
-  </si>
-  <si>
-    <t>ANZUELO</t>
-  </si>
-  <si>
-    <t>Codigo_1</t>
-  </si>
-  <si>
-    <t>Codigo_2</t>
-  </si>
-  <si>
-    <t>Codigo_3</t>
-  </si>
-  <si>
-    <t>Codigo_4</t>
   </si>
 </sst>
 </file>
@@ -596,7 +578,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:BH2"/>
+  <dimension ref="A1:BC2"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.28515625" bestFit="1" customWidth="1"/>
@@ -613,20 +595,18 @@
     <col min="12" max="12" width="38.28515625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="12.85546875" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="12.85546875" customWidth="1"/>
-    <col min="22" max="22" width="12" bestFit="1" customWidth="1"/>
-    <col min="44" max="44" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="45" max="45" width="27.140625" bestFit="1" customWidth="1"/>
-    <col min="46" max="46" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="47" max="47" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="48" max="48" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="50" max="50" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="52" max="52" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="54" max="54" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="59" max="59" width="13.28515625" customWidth="1"/>
+    <col min="39" max="39" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="27.140625" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="42" max="42" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="45" max="45" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="47" max="47" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="49" max="49" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="54" max="54" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -670,145 +650,130 @@
         <v>10</v>
       </c>
       <c r="O1" t="s">
-        <v>76</v>
+        <v>15</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="Q1" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="R1" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="S1" t="s">
-        <v>21</v>
+        <v>63</v>
       </c>
       <c r="T1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="U1" t="s">
-        <v>64</v>
+        <v>22</v>
       </c>
       <c r="V1" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="W1" t="s">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="X1" t="s">
-        <v>65</v>
+        <v>23</v>
       </c>
       <c r="Y1" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="Z1" t="s">
-        <v>23</v>
+        <v>66</v>
       </c>
       <c r="AA1" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="AB1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="AC1" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="AD1" t="s">
-        <v>31</v>
+        <v>67</v>
       </c>
       <c r="AE1" t="s">
-        <v>25</v>
+        <v>32</v>
       </c>
       <c r="AF1" t="s">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="AG1" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="AH1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="AI1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="AJ1" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="AK1" t="s">
-        <v>81</v>
+        <v>42</v>
       </c>
       <c r="AL1" t="s">
-        <v>28</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>68</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>33</v>
+        <v>43</v>
+      </c>
+      <c r="AM1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="AN1" s="2" t="s">
+        <v>47</v>
       </c>
       <c r="AO1" t="s">
-        <v>29</v>
+        <v>48</v>
       </c>
       <c r="AP1" t="s">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="AQ1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AR1" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="AS1" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>49</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>51</v>
       </c>
       <c r="AT1" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="AU1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AV1" t="s">
         <v>49</v>
       </c>
-      <c r="AV1" t="s">
-        <v>50</v>
-      </c>
       <c r="AW1" t="s">
+        <v>53</v>
+      </c>
+      <c r="AX1" t="s">
         <v>49</v>
       </c>
-      <c r="AX1" t="s">
-        <v>51</v>
-      </c>
       <c r="AY1" t="s">
-        <v>49</v>
+        <v>69</v>
       </c>
       <c r="AZ1" t="s">
-        <v>52</v>
+        <v>70</v>
       </c>
       <c r="BA1" t="s">
-        <v>49</v>
+        <v>71</v>
       </c>
       <c r="BB1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="BC1" t="s">
-        <v>49</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>69</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>70</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>71</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>72</v>
-      </c>
-      <c r="BH1" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:60" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>58</v>
       </c>
@@ -852,13 +817,13 @@
         <v>1</v>
       </c>
       <c r="O2" t="s">
-        <v>77</v>
-      </c>
-      <c r="P2" t="s">
         <v>38</v>
       </c>
+      <c r="Q2" t="s">
+        <v>19</v>
+      </c>
       <c r="R2" t="s">
-        <v>19</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
         <v>34</v>
@@ -867,111 +832,96 @@
         <v>34</v>
       </c>
       <c r="U2" t="s">
-        <v>34</v>
-      </c>
-      <c r="V2">
-        <v>34647567567</v>
-      </c>
-      <c r="W2" t="s">
         <v>35</v>
       </c>
-      <c r="X2" t="s">
+      <c r="V2" t="s">
         <v>11</v>
       </c>
-      <c r="Y2">
+      <c r="W2">
         <v>15</v>
       </c>
-      <c r="Z2">
+      <c r="X2">
         <v>2.5</v>
       </c>
+      <c r="Y2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Z2" t="s">
+        <v>74</v>
+      </c>
       <c r="AA2">
-        <v>5234646457</v>
-      </c>
-      <c r="AB2" t="s">
-        <v>36</v>
+        <v>13</v>
+      </c>
+      <c r="AB2">
+        <v>2.6</v>
       </c>
       <c r="AC2" t="s">
-        <v>74</v>
-      </c>
-      <c r="AD2">
+        <v>37</v>
+      </c>
+      <c r="AD2" t="s">
+        <v>11</v>
+      </c>
+      <c r="AE2">
+        <v>16</v>
+      </c>
+      <c r="AF2">
+        <v>2.7</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>39</v>
+      </c>
+      <c r="AH2" t="s">
+        <v>75</v>
+      </c>
+      <c r="AI2">
+        <v>20</v>
+      </c>
+      <c r="AJ2">
+        <v>2.6</v>
+      </c>
+      <c r="AK2">
         <v>13</v>
       </c>
-      <c r="AE2">
-        <v>2.6</v>
-      </c>
-      <c r="AF2">
-        <v>4534535354</v>
-      </c>
-      <c r="AG2" t="s">
-        <v>37</v>
-      </c>
-      <c r="AH2" t="s">
-        <v>11</v>
-      </c>
-      <c r="AI2">
-        <v>16</v>
-      </c>
-      <c r="AJ2">
-        <v>2.7</v>
-      </c>
-      <c r="AK2">
-        <v>534534534</v>
-      </c>
       <c r="AL2" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="AM2" t="s">
-        <v>75</v>
-      </c>
-      <c r="AN2">
-        <v>20</v>
-      </c>
-      <c r="AO2">
-        <v>2.6</v>
+        <v>46</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>45141</v>
+      </c>
+      <c r="AO2" t="s">
+        <v>54</v>
       </c>
       <c r="AP2">
+        <v>5</v>
+      </c>
+      <c r="AQ2" t="s">
+        <v>55</v>
+      </c>
+      <c r="AR2">
+        <v>3</v>
+      </c>
+      <c r="AS2" t="s">
+        <v>56</v>
+      </c>
+      <c r="AT2">
         <v>13</v>
       </c>
-      <c r="AQ2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AR2" t="s">
-        <v>46</v>
-      </c>
-      <c r="AS2" s="1">
-        <v>45141</v>
-      </c>
-      <c r="AT2" t="s">
-        <v>54</v>
-      </c>
-      <c r="AU2">
-        <v>5</v>
-      </c>
-      <c r="AV2" t="s">
-        <v>55</v>
-      </c>
-      <c r="AW2">
-        <v>3</v>
-      </c>
-      <c r="AX2" t="s">
-        <v>56</v>
-      </c>
-      <c r="AY2">
-        <v>13</v>
-      </c>
-      <c r="BD2" t="s">
+      <c r="AY2" t="s">
         <v>62</v>
       </c>
-      <c r="BE2" t="s">
+      <c r="AZ2" t="s">
         <v>59</v>
       </c>
-      <c r="BF2" t="s">
+      <c r="BA2" t="s">
         <v>60</v>
       </c>
-      <c r="BG2" t="s">
+      <c r="BB2" t="s">
         <v>61</v>
       </c>
-      <c r="BH2">
+      <c r="BC2">
         <v>10</v>
       </c>
     </row>

</xml_diff>